<commit_message>
Documentação SA - 1
Realizada o inicio da primeira parte da documentação da SA. Além de atualizar a planilha.
</commit_message>
<xml_diff>
--- a/CRONOGRAMA ENTREGA SA - 2026.xlsx
+++ b/CRONOGRAMA ENTREGA SA - 2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme_pacheco151\Documents\GitHub\Aula_HTML\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme_pacheco151\Documents\GitHub\SA_Padaria\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D37EA0F-7A85-41CF-A173-1B806B1B970E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD1C50D6-5A2C-4206-9635-E2D16FA0449C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -989,7 +989,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="83">
   <si>
     <t>Cronograma de Entregas</t>
   </si>
@@ -2691,14 +2691,22 @@
       <c r="B4" s="40" t="s">
         <v>76</v>
       </c>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
+      <c r="C4" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>82</v>
+      </c>
       <c r="E4" s="13"/>
       <c r="F4" s="20"/>
       <c r="G4" s="13"/>
       <c r="H4" s="20"/>
-      <c r="I4" s="13"/>
-      <c r="J4" s="13"/>
+      <c r="I4" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>82</v>
+      </c>
       <c r="K4" s="13"/>
       <c r="L4" s="13"/>
       <c r="M4" s="13"/>
@@ -2707,9 +2715,15 @@
       <c r="P4" s="13"/>
       <c r="Q4" s="13"/>
       <c r="R4" s="13"/>
-      <c r="S4" s="13"/>
-      <c r="T4" s="13"/>
-      <c r="U4" s="13"/>
+      <c r="S4" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="T4" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="U4" s="13" t="s">
+        <v>82</v>
+      </c>
       <c r="V4" s="13"/>
       <c r="W4" s="13"/>
       <c r="X4" s="13"/>
@@ -3511,6 +3525,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101002A2853F13A3D7249A14FECCC3E4AB7E9" ma:contentTypeVersion="2" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="1cd358d7cfd62764d24fa1fe544b7873">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c068192a-5874-45e4-b7bf-bdcfcd196c34" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b46b875ef662ca906f1891be54ed35c2" ns2:_="">
     <xsd:import namespace="c068192a-5874-45e4-b7bf-bdcfcd196c34"/>
@@ -3642,22 +3671,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6C7E75C-3607-440A-8310-E06F05988316}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="c068192a-5874-45e4-b7bf-bdcfcd196c34"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA18C466-A113-47F6-8297-47F116471958}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D5D11E7-FAB8-49EB-B26B-2285E2D60017}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3673,28 +3711,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA18C466-A113-47F6-8297-47F116471958}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6C7E75C-3607-440A-8310-E06F05988316}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="c068192a-5874-45e4-b7bf-bdcfcd196c34"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Documentação SA - 2
Atualizado a documentação da SA, adicionando a introdução.
</commit_message>
<xml_diff>
--- a/CRONOGRAMA ENTREGA SA - 2026.xlsx
+++ b/CRONOGRAMA ENTREGA SA - 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme_pacheco151\Documents\GitHub\SA_Padaria\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD1C50D6-5A2C-4206-9635-E2D16FA0449C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACD62A14-C5B1-4FC9-A096-65F0F69B1C9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DATA_Entrega_ITENS" sheetId="2" r:id="rId1"/>
@@ -989,7 +989,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="83">
   <si>
     <t>Cronograma de Entregas</t>
   </si>
@@ -2697,7 +2697,9 @@
       <c r="D4" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="E4" s="13"/>
+      <c r="E4" s="13" t="s">
+        <v>82</v>
+      </c>
       <c r="F4" s="20"/>
       <c r="G4" s="13"/>
       <c r="H4" s="20"/>
@@ -2713,7 +2715,9 @@
       <c r="N4" s="13"/>
       <c r="O4" s="13"/>
       <c r="P4" s="13"/>
-      <c r="Q4" s="13"/>
+      <c r="Q4" s="13" t="s">
+        <v>82</v>
+      </c>
       <c r="R4" s="13"/>
       <c r="S4" s="13" t="s">
         <v>82</v>

</xml_diff>